<commit_message>
Update data excel terbaru
</commit_message>
<xml_diff>
--- a/data_sq.xlsx
+++ b/data_sq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ali\belajar python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7B272E-8243-4530-AED4-CD30CCD1D303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507B989F-4A9F-4180-B843-5715A7D02155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$1173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$1207</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -85735,7 +85735,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U1173" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:U1207" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>